<commit_message>
fix captions and small things
</commit_message>
<xml_diff>
--- a/docs/springs_RH.xlsx
+++ b/docs/springs_RH.xlsx
@@ -1322,7 +1322,7 @@
         <v>186</v>
       </c>
       <c r="D7" s="29">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="30" t="s">
@@ -2141,7 +2141,7 @@
         <v>8</v>
       </c>
       <c r="C7" s="29">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D7" s="29">
         <v>188</v>

</xml_diff>

<commit_message>
update spring map and pc naming
</commit_message>
<xml_diff>
--- a/docs/springs_RH.xlsx
+++ b/docs/springs_RH.xlsx
@@ -128,10 +128,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="176" formatCode="0.0"/>
+    <numFmt numFmtId="177" formatCode="0.0"/>
+    <numFmt numFmtId="178" formatCode="0"/>
+    <numFmt numFmtId="179" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="37">
+  <fonts count="81">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -372,8 +375,275 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF667B91"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF667B91"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF667B91"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF667B91"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF195DB1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF667B91"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF667B91"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF195DB1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF667B91"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF667B91"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF667B91"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF283C50"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF667B91"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF667B91"/>
+      <name val="Microsoft YaHei"/>
+    </font>
   </fonts>
-  <fills count="36">
+  <fills count="76">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -550,8 +820,204 @@
         <fgColor rgb="FFF5F7FA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF31475E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF31475E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDF2F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF31475E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF31475E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDF2F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF31475E"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="33">
+  <borders count="66">
     <border>
       <left/>
       <right/>
@@ -827,11 +1293,287 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="36" borderId="33"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -944,6 +1686,187 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="36" borderId="33" xfId="1"/>
+    <xf numFmtId="0" fontId="42" fillId="40" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="38" borderId="33" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="39" borderId="33" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="39" borderId="33" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="40" fillId="39" borderId="33" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="38" fillId="38" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="45" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="50" fillId="48" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="49" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="52" fillId="50" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="55" fillId="53" borderId="47" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="54" borderId="48" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="57" fillId="55" borderId="49" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="60" fillId="58" borderId="52" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="61" fillId="59" borderId="53" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="60" borderId="54" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="61" borderId="55" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="64" fillId="62" borderId="56" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="65" fillId="63" borderId="57" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="64" borderId="58" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="69" fillId="67" borderId="61" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="70" fillId="68" borderId="62" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="71" fillId="69" borderId="63" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="70" borderId="64" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="73" fillId="71" borderId="65" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="41" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="42" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="43" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="44" borderId="38" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="46" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="47" borderId="41" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="39" borderId="33" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="53" fillId="51" borderId="45" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="52" borderId="46" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="65" borderId="59" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="66" borderId="60" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="56" borderId="50" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="57" borderId="51" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="38" borderId="33" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="36" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="74" fillId="36" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="72" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="75" fillId="72" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="73" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="73" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="73" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="74" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="74" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="74" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="75" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="75" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="76" fillId="75" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="76" fillId="75" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="75" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="78" fillId="74" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="78" fillId="73" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="74" fillId="74" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="74" fillId="73" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="74" fillId="73" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="74" fillId="74" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="36" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="80" fillId="36" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1583,7 +2506,7 @@
         <v>34</v>
       </c>
       <c r="G25" s="15">
-        <v>341.18265644791148</v>
+        <v>344.1826564479115</v>
       </c>
       <c r="H25" s="16" t="s">
         <v>13</v>
@@ -1606,7 +2529,7 @@
         <v>39</v>
       </c>
       <c r="G26" s="19">
-        <v>332.18265644791143</v>
+        <v>335.1826564479114</v>
       </c>
       <c r="H26" s="20" t="s">
         <v>14</v>
@@ -1629,7 +2552,7 @@
         <v>44</v>
       </c>
       <c r="G27" s="15">
-        <v>325.18265644791143</v>
+        <v>328.1826564479114</v>
       </c>
       <c r="H27" s="17" t="s">
         <v>14</v>
@@ -1652,7 +2575,7 @@
         <v>49</v>
       </c>
       <c r="G28" s="19">
-        <v>319.18265644791143</v>
+        <v>322.1826564479114</v>
       </c>
       <c r="H28" s="20" t="s">
         <v>14</v>
@@ -1675,7 +2598,7 @@
         <v>54</v>
       </c>
       <c r="G29" s="15">
-        <v>315.18265644791143</v>
+        <v>318.1826564479114</v>
       </c>
       <c r="H29" s="17" t="s">
         <v>14</v>
@@ -1698,7 +2621,7 @@
         <v>59</v>
       </c>
       <c r="G30" s="19">
-        <v>311.18265644791148</v>
+        <v>314.1826564479114</v>
       </c>
       <c r="H30" s="20" t="s">
         <v>14</v>
@@ -1751,126 +2674,184 @@
       <c r="H34" s="32"/>
       <c r="I34" s="2"/>
     </row>
-    <row r="35" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A35" s="2"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="2"/>
-    </row>
-    <row r="36" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A36" s="2"/>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
-      <c r="H36" s="32"/>
-      <c r="I36" s="2"/>
-    </row>
-    <row r="37" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A37" s="2"/>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="32"/>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="32"/>
-      <c r="I37" s="2"/>
-    </row>
-    <row r="38" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A38" s="2"/>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="32"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
-      <c r="H38" s="32"/>
-      <c r="I38" s="2"/>
-    </row>
-    <row r="39" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A39" s="2"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="2"/>
-    </row>
-    <row r="40" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A40" s="2"/>
-      <c r="B40" s="32"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="32"/>
-      <c r="E40" s="32"/>
-      <c r="F40" s="32"/>
-      <c r="G40" s="32"/>
-      <c r="H40" s="32"/>
-      <c r="I40" s="2"/>
-    </row>
-    <row r="41" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A41" s="2"/>
-      <c r="B41" s="32"/>
-      <c r="C41" s="32"/>
-      <c r="D41" s="32"/>
-      <c r="E41" s="32"/>
-      <c r="F41" s="32"/>
-      <c r="G41" s="32"/>
-      <c r="H41" s="32"/>
-      <c r="I41" s="2"/>
-    </row>
-    <row r="42" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A42" s="2"/>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
-      <c r="H42" s="32"/>
-      <c r="I42" s="2"/>
-    </row>
-    <row r="43" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A43" s="2"/>
-      <c r="B43" s="4"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
-      <c r="I43" s="2"/>
-    </row>
-    <row r="44" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A44" s="2"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-      <c r="I44" s="2"/>
-    </row>
-    <row r="45" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A45" s="2"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="2"/>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="42"/>
+      <c r="B35" s="83" t="str">
+        <v>Weight distribution · 重量分布</v>
+      </c>
+      <c r="C35" s="83"/>
+      <c r="D35" s="83"/>
+      <c r="E35" s="83"/>
+      <c r="F35" s="83"/>
+      <c r="G35" s="83"/>
+      <c r="H35" s="83"/>
+      <c r="I35" s="42"/>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="42"/>
+      <c r="B36" s="94" t="str">
+        <v>项目</v>
+      </c>
+      <c r="C36" s="94"/>
+      <c r="D36" s="94"/>
+      <c r="E36" s="93" t="str">
+        <v>Gravel</v>
+      </c>
+      <c r="F36" s="93"/>
+      <c r="G36" s="93" t="str">
+        <v>Tarmac</v>
+      </c>
+      <c r="H36" s="93"/>
+      <c r="I36" s="42"/>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="42"/>
+      <c r="B37" s="95" t="str">
+        <v>整车总重 (kg)</v>
+      </c>
+      <c r="C37" s="95"/>
+      <c r="D37" s="95"/>
+      <c r="E37" s="97" t="n">
+        <v>1390</v>
+      </c>
+      <c r="F37" s="97"/>
+      <c r="G37" s="97" t="n">
+        <v>1390</v>
+      </c>
+      <c r="H37" s="97"/>
+      <c r="I37" s="42"/>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="42"/>
+      <c r="B38" s="96" t="str">
+        <v>FL · 左前 (kg)</v>
+      </c>
+      <c r="C38" s="96"/>
+      <c r="D38" s="96"/>
+      <c r="E38" s="98" t="n">
+        <v>371</v>
+      </c>
+      <c r="F38" s="98"/>
+      <c r="G38" s="98" t="n">
+        <v>370</v>
+      </c>
+      <c r="H38" s="98"/>
+      <c r="I38" s="42"/>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="42"/>
+      <c r="B39" s="95" t="str">
+        <v>FR · 右前 (kg)</v>
+      </c>
+      <c r="C39" s="95"/>
+      <c r="D39" s="95"/>
+      <c r="E39" s="97" t="n">
+        <v>370</v>
+      </c>
+      <c r="F39" s="97"/>
+      <c r="G39" s="97" t="n">
+        <v>370</v>
+      </c>
+      <c r="H39" s="97"/>
+      <c r="I39" s="42"/>
+    </row>
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="42"/>
+      <c r="B40" s="96" t="str">
+        <v>RL · 左后 (kg)</v>
+      </c>
+      <c r="C40" s="96"/>
+      <c r="D40" s="96"/>
+      <c r="E40" s="98" t="n">
+        <v>324</v>
+      </c>
+      <c r="F40" s="98"/>
+      <c r="G40" s="98" t="n">
+        <v>326</v>
+      </c>
+      <c r="H40" s="98"/>
+      <c r="I40" s="42"/>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="42"/>
+      <c r="B41" s="95" t="str">
+        <v>RR · 右后 (kg)</v>
+      </c>
+      <c r="C41" s="95"/>
+      <c r="D41" s="95"/>
+      <c r="E41" s="97" t="n">
+        <v>325</v>
+      </c>
+      <c r="F41" s="97"/>
+      <c r="G41" s="97" t="n">
+        <v>325</v>
+      </c>
+      <c r="H41" s="97"/>
+      <c r="I41" s="42"/>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="42"/>
+      <c r="B42" s="96" t="str">
+        <v>前轴占比</v>
+      </c>
+      <c r="C42" s="96"/>
+      <c r="D42" s="96"/>
+      <c r="E42" s="99" t="n">
+        <f>SUM(E38:E39)/SUM(E38:E41)</f>
+        <v>0.5330935251798561</v>
+      </c>
+      <c r="F42" s="99"/>
+      <c r="G42" s="99" t="n">
+        <f>SUM(G38:G39)/SUM(G38:G41)</f>
+        <v>0.5319913731128685</v>
+      </c>
+      <c r="H42" s="99"/>
+      <c r="I42" s="42"/>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="42"/>
+      <c r="B43" s="95" t="str">
+        <v>后轴占比</v>
+      </c>
+      <c r="C43" s="95"/>
+      <c r="D43" s="95"/>
+      <c r="E43" s="100" t="n">
+        <f>SUM(E40:E41)/SUM(E38:E41)</f>
+        <v>0.46690647482014386</v>
+      </c>
+      <c r="F43" s="100"/>
+      <c r="G43" s="100" t="n">
+        <f>SUM(G40:G41)/SUM(G38:G41)</f>
+        <v>0.4680086268871316</v>
+      </c>
+      <c r="H43" s="100"/>
+      <c r="I43" s="42"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="42"/>
+      <c r="B44" s="101" t="str">
+        <v>2026-10-17</v>
+      </c>
+      <c r="C44" s="101"/>
+      <c r="D44" s="101"/>
+      <c r="E44" s="101"/>
+      <c r="F44" s="101"/>
+      <c r="G44" s="101"/>
+      <c r="H44" s="101"/>
+      <c r="I44" s="42"/>
+    </row>
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="42"/>
+      <c r="B45" s="102" t="str">
+        <v>轮荷为 UI 近似读数；前后比例按四轮读数计算。</v>
+      </c>
+      <c r="C45" s="102"/>
+      <c r="D45" s="102"/>
+      <c r="E45" s="102"/>
+      <c r="F45" s="102"/>
+      <c r="G45" s="102"/>
+      <c r="H45" s="102"/>
+      <c r="I45" s="42"/>
     </row>
     <row r="46" spans="1:9" ht="23.1" customHeight="1">
       <c r="A46" s="2"/>
@@ -1950,16 +2931,10 @@
       <c r="I52" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="B38:H38"/>
-    <mergeCell ref="B40:H40"/>
-    <mergeCell ref="B41:H41"/>
-    <mergeCell ref="B42:H42"/>
+  <mergeCells count="40">
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="B33:H33"/>
     <mergeCell ref="B34:H34"/>
-    <mergeCell ref="B36:H36"/>
-    <mergeCell ref="B37:H37"/>
     <mergeCell ref="B10:H10"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="F12:H12"/>
@@ -1970,6 +2945,33 @@
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="F6:G6"/>
+    <mergeCell ref="B35:H35"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="B44:H44"/>
+    <mergeCell ref="B45:H45"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2393,7 +3395,7 @@
         <v>37.5</v>
       </c>
       <c r="C25" s="15">
-        <v>339.93653951936574</v>
+        <v>345.93653951936574</v>
       </c>
       <c r="D25" s="16" t="s">
         <v>13</v>
@@ -2403,7 +3405,7 @@
         <v>32.5</v>
       </c>
       <c r="G25" s="15">
-        <v>341.18265644791148</v>
+        <v>347.1826564479115</v>
       </c>
       <c r="H25" s="16" t="s">
         <v>13</v>
@@ -2416,7 +3418,7 @@
         <v>42.5</v>
       </c>
       <c r="C26" s="19">
-        <v>329.93653951936574</v>
+        <v>335.93653951936574</v>
       </c>
       <c r="D26" s="20" t="s">
         <v>14</v>
@@ -2426,7 +3428,7 @@
         <v>37.5</v>
       </c>
       <c r="G26" s="19">
-        <v>331.18265644791143</v>
+        <v>337.1826564479114</v>
       </c>
       <c r="H26" s="20" t="s">
         <v>14</v>
@@ -2439,7 +3441,7 @@
         <v>47.5</v>
       </c>
       <c r="C27" s="15">
-        <v>322.93653951936574</v>
+        <v>328.93653951936574</v>
       </c>
       <c r="D27" s="17" t="s">
         <v>14</v>
@@ -2449,7 +3451,7 @@
         <v>42.5</v>
       </c>
       <c r="G27" s="15">
-        <v>323.18265644791143</v>
+        <v>329.1826564479114</v>
       </c>
       <c r="H27" s="17" t="s">
         <v>14</v>
@@ -2462,7 +3464,7 @@
         <v>52.5</v>
       </c>
       <c r="C28" s="19">
-        <v>315.93653951936574</v>
+        <v>321.93653951936574</v>
       </c>
       <c r="D28" s="20" t="s">
         <v>14</v>
@@ -2472,7 +3474,7 @@
         <v>47.5</v>
       </c>
       <c r="G28" s="19">
-        <v>318.18265644791143</v>
+        <v>324.1826564479114</v>
       </c>
       <c r="H28" s="20" t="s">
         <v>14</v>
@@ -2485,7 +3487,7 @@
         <v>57.5</v>
       </c>
       <c r="C29" s="15">
-        <v>310.93653951936574</v>
+        <v>316.93653951936574</v>
       </c>
       <c r="D29" s="17" t="s">
         <v>14</v>
@@ -2495,7 +3497,7 @@
         <v>52.5</v>
       </c>
       <c r="G29" s="15">
-        <v>313.18265644791143</v>
+        <v>319.1826564479114</v>
       </c>
       <c r="H29" s="17" t="s">
         <v>14</v>
@@ -2508,7 +3510,7 @@
         <v>62.5</v>
       </c>
       <c r="C30" s="19">
-        <v>306.93653951936579</v>
+        <v>312.93653951936574</v>
       </c>
       <c r="D30" s="20" t="s">
         <v>14</v>
@@ -2518,7 +3520,7 @@
         <v>57.5</v>
       </c>
       <c r="G30" s="19">
-        <v>310.18265644791148</v>
+        <v>316.1826564479114</v>
       </c>
       <c r="H30" s="20" t="s">
         <v>14</v>
@@ -2571,126 +3573,184 @@
       <c r="H34" s="32"/>
       <c r="I34" s="2"/>
     </row>
-    <row r="35" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A35" s="2"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="2"/>
-    </row>
-    <row r="36" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A36" s="2"/>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
-      <c r="H36" s="32"/>
-      <c r="I36" s="2"/>
-    </row>
-    <row r="37" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A37" s="2"/>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="32"/>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="32"/>
-      <c r="I37" s="2"/>
-    </row>
-    <row r="38" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A38" s="2"/>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="32"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
-      <c r="H38" s="32"/>
-      <c r="I38" s="2"/>
-    </row>
-    <row r="39" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A39" s="2"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="2"/>
-    </row>
-    <row r="40" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A40" s="2"/>
-      <c r="B40" s="32"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="32"/>
-      <c r="E40" s="32"/>
-      <c r="F40" s="32"/>
-      <c r="G40" s="32"/>
-      <c r="H40" s="32"/>
-      <c r="I40" s="2"/>
-    </row>
-    <row r="41" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A41" s="2"/>
-      <c r="B41" s="32"/>
-      <c r="C41" s="32"/>
-      <c r="D41" s="32"/>
-      <c r="E41" s="32"/>
-      <c r="F41" s="32"/>
-      <c r="G41" s="32"/>
-      <c r="H41" s="32"/>
-      <c r="I41" s="2"/>
-    </row>
-    <row r="42" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A42" s="2"/>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
-      <c r="H42" s="32"/>
-      <c r="I42" s="2"/>
-    </row>
-    <row r="43" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A43" s="2"/>
-      <c r="B43" s="4"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
-      <c r="I43" s="2"/>
-    </row>
-    <row r="44" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A44" s="2"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-      <c r="I44" s="2"/>
-    </row>
-    <row r="45" spans="1:9" ht="23.1" customHeight="1">
-      <c r="A45" s="2"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="2"/>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="42"/>
+      <c r="B35" s="83" t="str">
+        <v>Weight distribution · 重量分布</v>
+      </c>
+      <c r="C35" s="83"/>
+      <c r="D35" s="83"/>
+      <c r="E35" s="83"/>
+      <c r="F35" s="83"/>
+      <c r="G35" s="83"/>
+      <c r="H35" s="83"/>
+      <c r="I35" s="42"/>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="42"/>
+      <c r="B36" s="94" t="str">
+        <v>项目</v>
+      </c>
+      <c r="C36" s="94"/>
+      <c r="D36" s="94"/>
+      <c r="E36" s="93" t="str">
+        <v>Gravel</v>
+      </c>
+      <c r="F36" s="93"/>
+      <c r="G36" s="93" t="str">
+        <v>Tarmac</v>
+      </c>
+      <c r="H36" s="93"/>
+      <c r="I36" s="42"/>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="42"/>
+      <c r="B37" s="95" t="str">
+        <v>整车总重 (kg)</v>
+      </c>
+      <c r="C37" s="95"/>
+      <c r="D37" s="95"/>
+      <c r="E37" s="97" t="n">
+        <v>1420</v>
+      </c>
+      <c r="F37" s="97"/>
+      <c r="G37" s="97" t="n">
+        <v>1420</v>
+      </c>
+      <c r="H37" s="97"/>
+      <c r="I37" s="42"/>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="42"/>
+      <c r="B38" s="96" t="str">
+        <v>FL · 左前 (kg)</v>
+      </c>
+      <c r="C38" s="96"/>
+      <c r="D38" s="96"/>
+      <c r="E38" s="98" t="n">
+        <v>389</v>
+      </c>
+      <c r="F38" s="98"/>
+      <c r="G38" s="98" t="n">
+        <v>388</v>
+      </c>
+      <c r="H38" s="98"/>
+      <c r="I38" s="42"/>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="42"/>
+      <c r="B39" s="95" t="str">
+        <v>FR · 右前 (kg)</v>
+      </c>
+      <c r="C39" s="95"/>
+      <c r="D39" s="95"/>
+      <c r="E39" s="97" t="n">
+        <v>388</v>
+      </c>
+      <c r="F39" s="97"/>
+      <c r="G39" s="97" t="n">
+        <v>388</v>
+      </c>
+      <c r="H39" s="97"/>
+      <c r="I39" s="42"/>
+    </row>
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="42"/>
+      <c r="B40" s="96" t="str">
+        <v>RL · 左后 (kg)</v>
+      </c>
+      <c r="C40" s="96"/>
+      <c r="D40" s="96"/>
+      <c r="E40" s="98" t="n">
+        <v>322</v>
+      </c>
+      <c r="F40" s="98"/>
+      <c r="G40" s="98" t="n">
+        <v>322</v>
+      </c>
+      <c r="H40" s="98"/>
+      <c r="I40" s="42"/>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="42"/>
+      <c r="B41" s="95" t="str">
+        <v>RR · 右后 (kg)</v>
+      </c>
+      <c r="C41" s="95"/>
+      <c r="D41" s="95"/>
+      <c r="E41" s="97" t="n">
+        <v>321</v>
+      </c>
+      <c r="F41" s="97"/>
+      <c r="G41" s="97" t="n">
+        <v>322</v>
+      </c>
+      <c r="H41" s="97"/>
+      <c r="I41" s="42"/>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="42"/>
+      <c r="B42" s="96" t="str">
+        <v>前轴占比</v>
+      </c>
+      <c r="C42" s="96"/>
+      <c r="D42" s="96"/>
+      <c r="E42" s="99" t="n">
+        <f>SUM(E38:E39)/SUM(E38:E41)</f>
+        <v>0.5471830985915493</v>
+      </c>
+      <c r="F42" s="99"/>
+      <c r="G42" s="99" t="n">
+        <f>SUM(G38:G39)/SUM(G38:G41)</f>
+        <v>0.5464788732394367</v>
+      </c>
+      <c r="H42" s="99"/>
+      <c r="I42" s="42"/>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="42"/>
+      <c r="B43" s="95" t="str">
+        <v>后轴占比</v>
+      </c>
+      <c r="C43" s="95"/>
+      <c r="D43" s="95"/>
+      <c r="E43" s="100" t="n">
+        <f>SUM(E40:E41)/SUM(E38:E41)</f>
+        <v>0.4528169014084507</v>
+      </c>
+      <c r="F43" s="100"/>
+      <c r="G43" s="100" t="n">
+        <f>SUM(G40:G41)/SUM(G38:G41)</f>
+        <v>0.4535211267605634</v>
+      </c>
+      <c r="H43" s="100"/>
+      <c r="I43" s="42"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="42"/>
+      <c r="B44" s="101" t="str">
+        <v>2026-10-17</v>
+      </c>
+      <c r="C44" s="101"/>
+      <c r="D44" s="101"/>
+      <c r="E44" s="101"/>
+      <c r="F44" s="101"/>
+      <c r="G44" s="101"/>
+      <c r="H44" s="101"/>
+      <c r="I44" s="42"/>
+    </row>
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="42"/>
+      <c r="B45" s="102" t="str">
+        <v>轮荷为 UI 近似读数；前后比例按四轮读数计算。</v>
+      </c>
+      <c r="C45" s="102"/>
+      <c r="D45" s="102"/>
+      <c r="E45" s="102"/>
+      <c r="F45" s="102"/>
+      <c r="G45" s="102"/>
+      <c r="H45" s="102"/>
+      <c r="I45" s="42"/>
     </row>
     <row r="46" spans="1:9" ht="23.1" customHeight="1">
       <c r="A46" s="2"/>
@@ -2770,16 +3830,10 @@
       <c r="I52" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="B38:H38"/>
-    <mergeCell ref="B40:H40"/>
-    <mergeCell ref="B41:H41"/>
-    <mergeCell ref="B42:H42"/>
+  <mergeCells count="40">
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="B33:H33"/>
     <mergeCell ref="B34:H34"/>
-    <mergeCell ref="B36:H36"/>
-    <mergeCell ref="B37:H37"/>
     <mergeCell ref="B10:H10"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="F12:H12"/>
@@ -2790,6 +3844,33 @@
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="F6:G6"/>
+    <mergeCell ref="B35:H35"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="B44:H44"/>
+    <mergeCell ref="B45:H45"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>